<commit_message>
Add explainable risk scoring and risk classification
</commit_message>
<xml_diff>
--- a/output/audit_risk_report.xlsx
+++ b/output/audit_risk_report.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G11"/>
+  <dimension ref="A1:I11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -456,6 +456,16 @@
           <t>Risk_Score</t>
         </is>
       </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Risk_Reasons</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Risk_Level</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -485,6 +495,16 @@
       <c r="G2" t="n">
         <v>3</v>
       </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Weekend Posting; Round Dollar; High Value; </t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -514,6 +534,16 @@
       <c r="G3" t="n">
         <v>2</v>
       </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Round Dollar; High Value; </t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -543,6 +573,16 @@
       <c r="G4" t="n">
         <v>2</v>
       </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Round Dollar; High Value; </t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -572,6 +612,16 @@
       <c r="G5" t="n">
         <v>2</v>
       </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Weekend Posting; Round Dollar; </t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -601,6 +651,16 @@
       <c r="G6" t="n">
         <v>2</v>
       </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Weekend Posting; High Value; </t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -630,6 +690,16 @@
       <c r="G7" t="n">
         <v>1</v>
       </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Potential Duplicate; </t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -659,6 +729,16 @@
       <c r="G8" t="n">
         <v>1</v>
       </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Potential Duplicate; </t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -688,6 +768,12 @@
       <c r="G9" t="n">
         <v>0</v>
       </c>
+      <c r="H9" t="inlineStr"/>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -717,6 +803,12 @@
       <c r="G10" t="n">
         <v>0</v>
       </c>
+      <c r="H10" t="inlineStr"/>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -745,6 +837,12 @@
       </c>
       <c r="G11" t="n">
         <v>0</v>
+      </c>
+      <c r="H11" t="inlineStr"/>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add audit configuration and validation controls
</commit_message>
<xml_diff>
--- a/output/audit_risk_report.xlsx
+++ b/output/audit_risk_report.xlsx
@@ -493,7 +493,7 @@
         </is>
       </c>
       <c r="G2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
@@ -532,7 +532,7 @@
         </is>
       </c>
       <c r="G3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
@@ -541,7 +541,7 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -571,7 +571,7 @@
         </is>
       </c>
       <c r="G4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
@@ -580,92 +580,92 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>JE003</t>
+          <t>JE004</t>
         </is>
       </c>
       <c r="B5" s="1" t="n">
-        <v>46270</v>
+        <v>46271</v>
       </c>
       <c r="C5" t="n">
-        <v>6100</v>
+        <v>5200</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Office Supplies</t>
+          <t>Equipment Repair</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>1000</v>
+        <v>8750</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>SMITH</t>
+          <t>ADMIN</t>
         </is>
       </c>
       <c r="G5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Weekend Posting; Round Dollar; </t>
+          <t xml:space="preserve">Weekend Posting; High Value; </t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>JE004</t>
+          <t>JE006</t>
         </is>
       </c>
       <c r="B6" s="1" t="n">
-        <v>46271</v>
+        <v>46273</v>
       </c>
       <c r="C6" t="n">
-        <v>5200</v>
+        <v>4100</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Equipment Repair</t>
+          <t>Customer Payment</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>8750</v>
+        <v>2500</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>ADMIN</t>
+          <t>WILLIAMS</t>
         </is>
       </c>
       <c r="G6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Weekend Posting; High Value; </t>
+          <t xml:space="preserve">Potential Duplicate; </t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>JE006</t>
+          <t>JE005</t>
         </is>
       </c>
       <c r="B7" s="1" t="n">
@@ -688,7 +688,7 @@
         </is>
       </c>
       <c r="G7" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
@@ -697,41 +697,41 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>JE005</t>
+          <t>JE003</t>
         </is>
       </c>
       <c r="B8" s="1" t="n">
-        <v>46273</v>
+        <v>46270</v>
       </c>
       <c r="C8" t="n">
-        <v>4100</v>
+        <v>6100</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Customer Payment</t>
+          <t>Office Supplies</t>
         </is>
       </c>
       <c r="E8" t="n">
-        <v>2500</v>
+        <v>1000</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>WILLIAMS</t>
+          <t>SMITH</t>
         </is>
       </c>
       <c r="G8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Potential Duplicate; </t>
+          <t xml:space="preserve">Weekend Posting; Round Dollar; </t>
         </is>
       </c>
       <c r="I8" t="inlineStr">

</xml_diff>